<commit_message>
Add SUAPE specials flow and manual ONE/ZIM carrier support
</commit_message>
<xml_diff>
--- a/artifacts/input/cma_jobs.xlsx
+++ b/artifacts/input/cma_jobs.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D223"/>
+  <dimension ref="A1:D254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37.28515625" customWidth="1" min="1" max="1"/>
@@ -530,7 +530,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -590,7 +590,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -650,7 +650,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -710,7 +710,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -770,7 +770,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -830,7 +830,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -890,7 +890,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -950,7 +950,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1010,7 +1010,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -1070,7 +1070,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1130,7 +1130,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -1190,7 +1190,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1250,7 +1250,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -1310,7 +1310,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -1430,7 +1430,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1490,7 +1490,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -1550,7 +1550,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -1610,7 +1610,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -1670,7 +1670,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -1730,7 +1730,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -1790,7 +1790,7 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -1850,7 +1850,7 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -1910,7 +1910,7 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -1970,7 +1970,7 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
@@ -2030,7 +2030,7 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -2090,7 +2090,7 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -2150,7 +2150,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -2210,7 +2210,7 @@
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
@@ -2270,7 +2270,7 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -2330,7 +2330,7 @@
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
@@ -2390,7 +2390,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -2450,7 +2450,7 @@
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
@@ -2510,7 +2510,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -2570,7 +2570,7 @@
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
@@ -2630,7 +2630,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -2730,7 +2730,7 @@
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
@@ -2846,7 +2846,7 @@
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
@@ -2906,7 +2906,7 @@
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
@@ -2966,7 +2966,7 @@
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
@@ -3026,7 +3026,7 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
@@ -3086,7 +3086,7 @@
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
@@ -3206,7 +3206,7 @@
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
@@ -3266,7 +3266,7 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -3326,7 +3326,7 @@
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
@@ -3386,7 +3386,7 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
@@ -3446,7 +3446,7 @@
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
@@ -3506,7 +3506,7 @@
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
@@ -3566,7 +3566,7 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
@@ -3686,7 +3686,7 @@
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
@@ -3806,7 +3806,7 @@
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
@@ -3926,7 +3926,7 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
@@ -3986,7 +3986,7 @@
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
@@ -4046,7 +4046,7 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
@@ -4106,7 +4106,7 @@
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
@@ -4166,7 +4166,7 @@
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
@@ -4226,7 +4226,7 @@
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B187" s="3" t="inlineStr">
@@ -4346,7 +4346,7 @@
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B193" s="3" t="inlineStr">
@@ -4406,7 +4406,7 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
@@ -4466,7 +4466,7 @@
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B199" s="3" t="inlineStr">
@@ -4526,7 +4526,7 @@
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
@@ -4586,7 +4586,7 @@
     <row r="205">
       <c r="A205" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B205" s="3" t="inlineStr">
@@ -4686,7 +4686,7 @@
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
@@ -4726,7 +4726,7 @@
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
@@ -4846,7 +4846,7 @@
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
@@ -4906,7 +4906,7 @@
     <row r="221">
       <c r="A221" s="3" t="inlineStr">
         <is>
-          <t>Itajai (Santa Catarina), Brazil</t>
+          <t>BRITJ</t>
         </is>
       </c>
       <c r="B221" s="3" t="inlineStr">
@@ -4961,6 +4961,626 @@
       </c>
       <c r="D223" s="3" t="n">
         <v>224</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>BRITJ</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>CUMAR</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Mariel, Cuba</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>BRSSA</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>CUMAR</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Mariel, Cuba</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>BRSSZ</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>CUMAR</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Mariel, Cuba</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>BRITJ</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>PAMIT</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Manzanillo (Colima), Mexico</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>BRSSA</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>PAMIT</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Manzanillo (Colima), Mexico</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>BRSSZ</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>PAMIT</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Manzanillo (Colima), Mexico</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>BRITJ</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>KYGCM</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Grand Cayman, Cayman Islands</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>BRSSA</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>KYGCM</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Grand Cayman, Cayman Islands</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>BRSSZ</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>KYGCM</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Grand Cayman, Cayman Islands</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>KNBAS</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Basseterre, St Kitts-Nevis</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>BBBGI</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Bridgetown, Barbados</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>VCCRP</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Campden Park, Saint Vincent and the Grenadines</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>DOCAU</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Caucedo, Dominican Republic</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>PACTB</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Cristobal, Panama</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>BSFPO</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Freeport, Bahamas</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>AUGEE</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Georgetown, Guyana</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>JMKIN</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Kingston, Jamaica</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>BQKRA</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>KRALENDIJK, BONAIRE</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>BSNAS</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Nassau, Bahamas</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>AWORJ</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Oranjestad, Aruba</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>SRPBM</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Paramaribo, Suriname</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>TTPOS</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Port of Spain-Trinidad, Trinidad and Tobago</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>VGRAD</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Road Town, Virgin Islands (Br.)</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>DMRSU</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Roseau, Dominica</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>GDSTG</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Saint George, Grenada</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>PRSJU</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>San Juan, Puerto Rico</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>AGSJO</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>St Johns, Antigua and Barbuda</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>ANWIL</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Willemstad, Curacao</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>CUMAR</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Mariel, Cuba</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>PAMIT</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Manzanillo (Colima), Mexico</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>BRSUA</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>KYGCM</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Grand Cayman, Cayman Islands</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add granite output flow and new route matrices
</commit_message>
<xml_diff>
--- a/artifacts/input/cma_jobs.xlsx
+++ b/artifacts/input/cma_jobs.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D254"/>
+  <dimension ref="A1:D260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37.28515625" customWidth="1" min="1" max="1"/>
@@ -5583,6 +5583,126 @@
         <v>255</v>
       </c>
     </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>BRVIX</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>MXATM</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Altamira (Tamaulipas), Mexico</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>BRVIX</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>MXVER</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Veracruz (Veracruz Llave), Mexico</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>BRVIX</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>PAMIT</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Manzanillo, Panama</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>BRVIX</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>DOCAU</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Caucedo, Dominican Republic</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>BRVIX</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>PRSJU</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>San Juan, Puerto Rico</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>BRVIX</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>COCTG</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Cartagena (Bolivar), Colombia</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>263</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D223">
     <sortState ref="A2:D223">

</xml_diff>